<commit_message>
Session 8: filter panel reorder + Filters header; word-wrap labels; Abundant Intelligences group
- Filter panel: Group → Program → Project → Categories order; "Filters" section header added
- SVG group labels word-wrap up to 3 lines (wrapLabel + svgWrappedLabel helpers)
- Added Abundant Intelligences group to AbTeC-Timeline-Data.xlsx (1203 rows)
- README.txt → README.md (full markdown)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/timeline-data/AbTeC-Timeline-Data.xlsx
+++ b/data/timeline-data/AbTeC-Timeline-Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jasonlocal/Documents/Coding-Experiments/Timeline/Timeline-JEL/data/timeline-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28CF3F7F-CCFE-DE40-A407-3DC97AAEA768}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64D083DF-5DC8-E64E-94FA-40E048C29609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4600" yWindow="500" windowWidth="33700" windowHeight="16940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6792,16 +6792,16 @@
     <t>https://abundant-intelligences.net/news/ef01/</t>
   </si>
   <si>
-    <t>Epistemological Foundations 01: Indigenous Theory and Methdology</t>
-  </si>
-  <si>
-    <t>Integrating Indigenous Knowledges with the knowledge systems that underlie AI research is fraught with epistemic challenges. Fundamental questions about what counts as knowledge, how we validate that knowledge, and how we act on it become acute when such different frameworks for engaging the world come into relationship with one another.</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=ca6OCK6ZYOM</t>
-  </si>
-  <si>
-    <t>https://abundant-intelligences.net/wp-content/uploads/2024/05/AbInt_People_Tuhiwai-Smith_2024.jpg</t>
+    <t>https://vimeo.com/1101324352?share=copy&amp;fl=sv&amp;fe=ci</t>
+  </si>
+  <si>
+    <t>Epistemological Foundations 02: Artificial Intelligence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A major goal of the Conversation Series is to address these discrepancies so as to synchronize expertise, methodologies, and goals that reside within the Abundant Intelligences Research Program. This conversation addressed how knowledge is constructed in AI, and how the shortcomings of the field can be remedied through Indigenous ways of knowing. </t>
+  </si>
+  <si>
+    <t>https://yoshuabengio.org/profile/</t>
   </si>
 </sst>
 </file>
@@ -8402,10 +8402,10 @@
         <v>2023</v>
       </c>
       <c r="B3" s="8">
+        <v>2</v>
+      </c>
+      <c r="C3" s="8">
         <v>12</v>
-      </c>
-      <c r="C3" s="8">
-        <v>13</v>
       </c>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -8417,13 +8417,13 @@
         <v>2137</v>
       </c>
       <c r="K3" s="12" t="s">
+        <v>2139</v>
+      </c>
+      <c r="L3" s="13" t="s">
+        <v>2140</v>
+      </c>
+      <c r="M3" s="14" t="s">
         <v>2138</v>
-      </c>
-      <c r="L3" s="13" t="s">
-        <v>2139</v>
-      </c>
-      <c r="M3" s="14" t="s">
-        <v>2140</v>
       </c>
       <c r="N3" s="7"/>
       <c r="O3" s="7"/>
@@ -54221,8 +54221,8 @@
     <hyperlink ref="J552" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000055020000}"/>
     <hyperlink ref="J553" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000056020000}"/>
     <hyperlink ref="J2" r:id="rId85" display="&lt;a href=&quot;http://skins.abtec.org/skins4.0/&quot;&gt;Skins 4.0&lt;/a&gt;" xr:uid="{C23EC51E-4914-AF4F-97A7-F47BB31C9E51}"/>
-    <hyperlink ref="M2" r:id="rId86" xr:uid="{77726E42-2015-3B4D-9663-430BB11ABC72}"/>
-    <hyperlink ref="M4" r:id="rId87" xr:uid="{C525E5F6-3A4F-4440-8AAB-4A497B07158E}"/>
+    <hyperlink ref="M4" r:id="rId86" xr:uid="{C525E5F6-3A4F-4440-8AAB-4A497B07158E}"/>
+    <hyperlink ref="M2" r:id="rId87" xr:uid="{77726E42-2015-3B4D-9663-430BB11ABC72}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>